<commit_message>
Added Ex2B_data_roundup.xlsx to week-01
</commit_message>
<xml_diff>
--- a/week-01/Ex2B_data_roundup.xlsx
+++ b/week-01/Ex2B_data_roundup.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sayaeedarashullahakr\Documents\DataAnalytics\week-01\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3E04CBA8-DCD4-44CF-93FC-1D7C02EF9AA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB4EAC4C-4AAA-4F49-AC13-0B6D84012AAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{632274E4-23F1-4D38-AE6F-84C997174C60}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="25">
   <si>
     <t>Name of data source</t>
   </si>
@@ -121,13 +121,16 @@
   <si>
     <t>You can use purchase history to see what you
  bought and how much have you spent</t>
+  </si>
+  <si>
+    <t>10-18-2026: No changes to the file updating the commit history.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -140,6 +143,14 @@
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -164,9 +175,11 @@
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -503,114 +516,120 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8CA7169C-CD30-47F2-8F97-DEC8154CBED9}">
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="24.88671875" customWidth="1"/>
+    <col min="1" max="1" width="28.6640625" customWidth="1"/>
     <col min="2" max="2" width="37" customWidth="1"/>
     <col min="3" max="3" width="33.77734375" customWidth="1"/>
     <col min="4" max="4" width="37.5546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>8</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
+      <c r="A2" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" t="s">
         <v>11</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
+      <c r="A3" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" t="s">
         <v>13</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="D3" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4" s="1" t="s">
+      <c r="A4" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" t="s">
         <v>14</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="D4" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="1" t="s">
+      <c r="A5" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="2" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6" s="1" t="s">
+      <c r="A6" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" t="s">
         <v>19</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="D6" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="33" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="1" t="s">
+      <c r="A7" t="s">
         <v>3</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="D7" s="2" t="s">
         <v>23</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="3" t="s">
+        <v>24</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>